<commit_message>
#22 Updated BOM files
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.2/BOM/eSpark-BOM-IoT-Speaker.xlsx
+++ b/Design Files/IoT-Speaker-v1.2/BOM/eSpark-BOM-IoT-Speaker.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="2 Boards" sheetId="2" r:id="rId1"/>
@@ -2276,7 +2276,7 @@
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -6595,7 +6595,7 @@
         <v>5</v>
       </c>
       <c r="N18" s="37">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O18" s="64" t="s">
         <v>161</v>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="Q18" s="38">
         <f>P18*N18</f>
-        <v>0.89600000000000002</v>
+        <v>0.44800000000000001</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="56"/>
@@ -9159,7 +9159,7 @@
       <c r="P64" s="81"/>
       <c r="Q64" s="48">
         <f>SUM(Q10:Q62)</f>
-        <v>191.21681999999998</v>
+        <v>190.76881999999998</v>
       </c>
       <c r="R64" s="45"/>
       <c r="S64" s="45"/>
@@ -9185,7 +9185,7 @@
       <c r="P65" s="81"/>
       <c r="Q65" s="48">
         <f>Q64/5</f>
-        <v>38.243364</v>
+        <v>38.153763999999995</v>
       </c>
       <c r="R65" s="10"/>
       <c r="S65" s="10"/>
@@ -10014,7 +10014,7 @@
         <v>50</v>
       </c>
       <c r="N18" s="37">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O18" s="64" t="s">
         <v>161</v>
@@ -10024,7 +10024,7 @@
       </c>
       <c r="Q18" s="38">
         <f>P18*N18</f>
-        <v>3.5859999999999999</v>
+        <v>1.9559999999999997</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="56"/>
@@ -12581,7 +12581,7 @@
       <c r="P64" s="81"/>
       <c r="Q64" s="48">
         <f>SUM(Q10:Q62)</f>
-        <v>1325.91463</v>
+        <v>1324.2846299999999</v>
       </c>
       <c r="R64" s="45"/>
       <c r="S64" s="45"/>
@@ -12607,7 +12607,7 @@
       <c r="P65" s="81"/>
       <c r="Q65" s="48">
         <f>Q64/50</f>
-        <v>26.518292599999999</v>
+        <v>26.485692599999997</v>
       </c>
       <c r="R65" s="10"/>
       <c r="S65" s="10"/>

</xml_diff>

<commit_message>
BOM sum issue fix #22
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.2/BOM/eSpark-BOM-IoT-Speaker.xlsx
+++ b/Design Files/IoT-Speaker-v1.2/BOM/eSpark-BOM-IoT-Speaker.xlsx
@@ -5,18 +5,18 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Speaker-v1.2\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Speaker-v1.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="2 Boards" sheetId="2" r:id="rId1"/>
     <sheet name="5 Boards" sheetId="1" r:id="rId2"/>
     <sheet name="50 Boards" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -1052,7 +1052,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1573,7 +1573,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1822,6 +1822,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1866,7 +1867,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1920,7 +1921,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1974,7 +1975,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9158,8 +9159,8 @@
       <c r="O64" s="81"/>
       <c r="P64" s="81"/>
       <c r="Q64" s="48">
-        <f>SUM(Q10:Q62)</f>
-        <v>190.76881999999998</v>
+        <f>SUM(Q10:Q63)</f>
+        <v>194.06881999999999</v>
       </c>
       <c r="R64" s="45"/>
       <c r="S64" s="45"/>
@@ -9185,10 +9186,13 @@
       <c r="P65" s="81"/>
       <c r="Q65" s="48">
         <f>Q64/5</f>
-        <v>38.153763999999995</v>
+        <v>38.813763999999999</v>
       </c>
       <c r="R65" s="10"/>
       <c r="S65" s="10"/>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="Q68" s="90"/>
     </row>
     <row r="77" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="N77" s="67"/>
@@ -12580,8 +12584,8 @@
       <c r="O64" s="81"/>
       <c r="P64" s="81"/>
       <c r="Q64" s="48">
-        <f>SUM(Q10:Q62)</f>
-        <v>1324.2846299999999</v>
+        <f>SUM(Q10:Q63)</f>
+        <v>1357.2846299999999</v>
       </c>
       <c r="R64" s="45"/>
       <c r="S64" s="45"/>
@@ -12607,7 +12611,7 @@
       <c r="P65" s="81"/>
       <c r="Q65" s="48">
         <f>Q64/50</f>
-        <v>26.485692599999997</v>
+        <v>27.145692599999997</v>
       </c>
       <c r="R65" s="10"/>
       <c r="S65" s="10"/>

</xml_diff>